<commit_message>
Update onboarding labels and Aug 17-21 data
</commit_message>
<xml_diff>
--- a/data/数据源8.17-8.21.xlsx
+++ b/data/数据源8.17-8.21.xlsx
@@ -4604,10 +4604,10 @@
         <v>2</v>
       </c>
       <c r="M33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N33" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="O33">
         <v>0</v>

</xml_diff>